<commit_message>
Align import template columns with export catalog columns, auto-generate missing SKUs and link to barcode
</commit_message>
<xml_diff>
--- a/inventory_template.xlsx
+++ b/inventory_template.xlsx
@@ -401,7 +401,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name</v>
+        <v>Product Name</v>
       </c>
       <c r="B1" t="str">
         <v>SKU</v>
@@ -413,54 +413,54 @@
         <v>Category</v>
       </c>
       <c r="E1" t="str">
-        <v>Unit Price</v>
+        <v>Supplier</v>
       </c>
       <c r="F1" t="str">
-        <v>Cost Price</v>
+        <v>Cost Price (£)</v>
       </c>
       <c r="G1" t="str">
-        <v>Quantity On Hand</v>
+        <v>Retail Price (£)</v>
       </c>
       <c r="H1" t="str">
-        <v>Reorder Threshold</v>
+        <v>Stock Qty</v>
       </c>
       <c r="I1" t="str">
-        <v>Supplier</v>
+        <v>Reorder Level</v>
       </c>
       <c r="J1" t="str">
-        <v>Expiry Date (YYYY-MM-DD)</v>
+        <v>Expiry Date</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Organic Bananas 1kg</v>
+        <v>Fresh Organic Strawberries 400g</v>
       </c>
       <c r="B2" t="str">
-        <v>PRD-BAN-ORG</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>5000112637991</v>
+        <v>5000112637990</v>
       </c>
       <c r="D2" t="str">
         <v>Fruits &amp; Vegetables</v>
       </c>
       <c r="E2" t="str">
-        <v>1.89</v>
+        <v>Fresh Farms Ltd</v>
       </c>
       <c r="F2" t="str">
-        <v>0.95</v>
+        <v>1.50</v>
       </c>
       <c r="G2" t="str">
-        <v>80</v>
+        <v>2.99</v>
       </c>
       <c r="H2" t="str">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="I2" t="str">
-        <v>Fresh Farms Ltd</v>
+        <v>10</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-08-05</v>
+        <v>2026-08-10</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         <v>Dairy &amp; Eggs</v>
       </c>
       <c r="E3" t="str">
-        <v>1.55</v>
+        <v>Metro Wholesale</v>
       </c>
       <c r="F3" t="str">
         <v>0.85</v>
       </c>
       <c r="G3" t="str">
+        <v>1.55</v>
+      </c>
+      <c r="H3" t="str">
         <v>100</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>20</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Metro Wholesale</v>
       </c>
       <c r="J3" t="str">
         <v>2026-08-15</v>

</xml_diff>